<commit_message>
update logic and import file template for writing, matching question revision
</commit_message>
<xml_diff>
--- a/frontend/public/general_revision/MATCHING.xlsx
+++ b/frontend/public/general_revision/MATCHING.xlsx
@@ -399,64 +399,64 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B7"/>
   <cols>
-    <col min="1" max="1" width="55.83203125" customWidth="1"/>
-    <col min="2" max="2" width="45.83203125" customWidth="1"/>
+    <col min="1" max="1" width="28.83203125" customWidth="1"/>
+    <col min="2" max="2" width="32.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>left</v>
+        <v>Left</v>
       </c>
       <c r="B1" t="str">
-        <v>right</v>
+        <v>Right</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>[Bắt buộc] Vế trái (text hoặc URL ảnh)</v>
+        <v>(left item)</v>
       </c>
       <c r="B2" t="str">
-        <v>[Bắt buộc] Vế phải (text)</v>
+        <v>(right item)</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>a letter describing your character and ability to pay rent</v>
+        <v>Apple</v>
       </c>
       <c r="B3" t="str">
-        <v>a reference</v>
+        <v>A red fruit</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>houses and apartments that are for sale or rented out</v>
+        <v>Banana</v>
       </c>
       <c r="B4" t="str">
-        <v>real estate / property</v>
+        <v>A yellow fruit</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>a part of town where most buildings are houses or apartments</v>
+        <v>Carrot</v>
       </c>
       <c r="B5" t="str">
-        <v>a residential area</v>
+        <v>An orange vegetable</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>https://res.cloudinary.com/.../write_2.png</v>
+        <v>Dog</v>
       </c>
       <c r="B6" t="str">
-        <v>I love playing with my grandson.</v>
+        <v>A domestic animal</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>https://res.cloudinary.com/.../write_3.png</v>
+        <v>Cat</v>
       </c>
       <c r="B7" t="str">
-        <v>We are bringing up our children to work hard.</v>
+        <v>A feline animal</v>
       </c>
     </row>
   </sheetData>

</xml_diff>